<commit_message>
Agrega figura carga-deflexión y gráfico en la planilla
</commit_message>
<xml_diff>
--- a/analysis/analisis_viga.xlsx
+++ b/analysis/analisis_viga.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d92907fbc3d0b6c/Documents/Herramientas computacionales 2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d92907fbc3d0b6c/Documents/Herramientas computacionales 2/Hito 1 viga/analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="8_{3EA512AB-3D69-4FD8-A159-5C7BE8F45010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DCCE0A0-A710-409B-8951-68D8CE7713B4}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="8_{3EA512AB-3D69-4FD8-A159-5C7BE8F45010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2606D4CB-4016-4A2F-AB65-D32EC86B05F9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3FF4F9D9-3A17-4D22-98E0-7BB1BB8380C0}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametros " sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcCompleted="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -413,8 +413,1223 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-MX"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-CL"/>
+              <a:t>Carga</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" baseline="0"/>
+              <a:t>-deflexión en el centro de la luz</a:t>
+            </a:r>
+            <a:endParaRPr lang="es-CL"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CL"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Medida</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Parametros '!$B$12:$B$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>40</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Parametros '!$D$12:$D$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.26</c:v>
+                </c:pt>
+                <c:pt idx="2" formatCode="0.00">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.76</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.01</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.28</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.54</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.77</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.0499999999999998</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-C34E-4398-9BDA-BD74E2B18D7F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Teórica (Euler-Bernoulli)</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Parametros '!$B$12:$B$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>40</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Parametros '!$F$12:$F$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.24999999999999994</c:v>
+                </c:pt>
+                <c:pt idx="2" formatCode="0.00">
+                  <c:v>0.49999999999999989</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.74999999999999989</c:v>
+                </c:pt>
+                <c:pt idx="4" formatCode="0.00">
+                  <c:v>0.99999999999999978</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.2499999999999998</c:v>
+                </c:pt>
+                <c:pt idx="6" formatCode="0.00">
+                  <c:v>1.4999999999999998</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.7499999999999996</c:v>
+                </c:pt>
+                <c:pt idx="8" formatCode="0.00">
+                  <c:v>1.9999999999999996</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-C34E-4398-9BDA-BD74E2B18D7F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="79621551"/>
+        <c:axId val="1640809135"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="79621551"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="es-CL"/>
+                  <a:t>Carga</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="es-CL" baseline="0"/>
+                  <a:t> P (kN)</a:t>
+                </a:r>
+                <a:endParaRPr lang="es-CL"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="es-CL"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1640809135"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1640809135"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="es-CL"/>
+                  <a:t>Deflexión</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="es-CL" baseline="0"/>
+                  <a:t> en el centro (mm)</a:t>
+                </a:r>
+                <a:endParaRPr lang="es-CL"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="es-CL"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="79621551"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CL"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-CL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>205740</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>22860</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>179070</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6368B050-A367-3A89-5FE7-D120F606FC03}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1097,5 +2312,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Agrega verificaciones de δ/P y calculo a mano
</commit_message>
<xml_diff>
--- a/analysis/analisis_viga.xlsx
+++ b/analysis/analisis_viga.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d92907fbc3d0b6c/Documents/Herramientas computacionales 2/Hito 1 viga/analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="8_{3EA512AB-3D69-4FD8-A159-5C7BE8F45010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2606D4CB-4016-4A2F-AB65-D32EC86B05F9}"/>
+  <xr:revisionPtr revIDLastSave="151" documentId="8_{3EA512AB-3D69-4FD8-A159-5C7BE8F45010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2EF461EA-6E9A-4428-ADF7-A8045E44540A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3FF4F9D9-3A17-4D22-98E0-7BB1BB8380C0}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametros " sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" calcCompleted="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
   <si>
     <t>Longitud (L)</t>
   </si>
@@ -286,13 +286,146 @@
   <si>
     <t>Parámetro</t>
   </si>
+  <si>
+    <r>
+      <t>δ</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>medida</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / P (mm/kN)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>I = 0,2 * 0,4</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / 12 = 0,0010667 m</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>δ = 20000 * 4</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / (48 * 25x10</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>9</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> * 0,0010667) = 0,001 m = 1 mm</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Resultado de la planilla para 20 kN (mm) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coincide totalmente con el cálculo analítico </t>
+  </si>
+  <si>
+    <t>Verificación B: cálculo independiente (P=20kN)</t>
+  </si>
+  <si>
+    <t>Promedio de δ/P medido (mm/kN)</t>
+  </si>
+  <si>
+    <t>δ/P teórico (mm/kN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">δ/P varía entre 0,050 y 0,052 mm/kN: el comportamiento es lineal </t>
+  </si>
+  <si>
+    <t>Verificación A : cálculo de δ/P</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.00000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -368,7 +501,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -393,6 +526,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1595,16 +1735,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>205740</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>364490</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>11112</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>22860</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>179070</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>181610</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>171132</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1630,6 +1770,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1949,18 +2093,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1656554-2448-43E1-9F2A-FE109927343C}">
-  <dimension ref="B2:G26"/>
+  <dimension ref="B2:H42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="40.88671875" customWidth="1"/>
-    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="2" max="2" width="55.5546875" customWidth="1"/>
+    <col min="3" max="3" width="25.33203125" customWidth="1"/>
     <col min="4" max="4" width="22.44140625" customWidth="1"/>
     <col min="5" max="5" width="17.5546875" customWidth="1"/>
     <col min="6" max="6" width="19.33203125" customWidth="1"/>
     <col min="7" max="7" width="18.44140625" customWidth="1"/>
+    <col min="8" max="8" width="17.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B2" s="3" t="s">
         <v>26</v>
       </c>
@@ -1971,7 +2116,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B3" s="4" t="s">
         <v>0</v>
       </c>
@@ -1982,7 +2127,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
         <v>1</v>
       </c>
@@ -1993,7 +2138,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>2</v>
       </c>
@@ -2004,7 +2149,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B6" s="4" t="s">
         <v>16</v>
       </c>
@@ -2017,7 +2162,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="1"/>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B7" s="4" t="s">
         <v>9</v>
       </c>
@@ -2029,7 +2174,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="2:7" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:8" ht="16.2" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
         <v>6</v>
       </c>
@@ -2041,7 +2186,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" ht="15.6" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
         <v>10</v>
       </c>
@@ -2060,8 +2205,11 @@
       <c r="G11" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H11" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B12" s="4">
         <v>0</v>
       </c>
@@ -2084,8 +2232,12 @@
         <f>+IF(C12=0,"",(D12-F12)/F12)</f>
         <v/>
       </c>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H12" s="5" t="str">
+        <f>+IF(B12=0,"",D12/B12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B13" s="4">
         <v>5</v>
       </c>
@@ -2108,8 +2260,12 @@
         <f>+IF(C13=0,"",(D13-F13)/F13)</f>
         <v>4.0000000000000265E-2</v>
       </c>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H13" s="11">
+        <f t="shared" ref="H13:H20" si="2">+IF(B13=0,"",D13/B13)</f>
+        <v>5.2000000000000005E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B14" s="4">
         <v>10</v>
       </c>
@@ -2121,7 +2277,7 @@
         <v>0.5</v>
       </c>
       <c r="E14" s="9">
-        <f t="shared" ref="E14:E20" si="2">+C14*($C$3)^3/(48*$C$7*$C$8)</f>
+        <f t="shared" ref="E14:E20" si="3">+C14*($C$3)^3/(48*$C$7*$C$8)</f>
         <v>4.999999999999999E-4</v>
       </c>
       <c r="F14" s="8">
@@ -2129,11 +2285,15 @@
         <v>0.49999999999999989</v>
       </c>
       <c r="G14" s="7">
-        <f t="shared" ref="G14:G20" si="3">+IF(C14=0,"",(D14-F14)/F14)</f>
+        <f t="shared" ref="G14:G20" si="4">+IF(C14=0,"",(D14-F14)/F14)</f>
         <v>2.2204460492503136E-16</v>
       </c>
-    </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H14" s="11">
+        <f t="shared" si="2"/>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B15" s="4">
         <v>15</v>
       </c>
@@ -2145,7 +2305,7 @@
         <v>0.76</v>
       </c>
       <c r="E15" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>7.4999999999999991E-4</v>
       </c>
       <c r="F15" s="4">
@@ -2153,11 +2313,15 @@
         <v>0.74999999999999989</v>
       </c>
       <c r="G15" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.3333333333333496E-2</v>
       </c>
-    </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H15" s="11">
+        <f t="shared" si="2"/>
+        <v>5.0666666666666665E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B16" s="4">
         <v>20</v>
       </c>
@@ -2169,7 +2333,7 @@
         <v>1.01</v>
       </c>
       <c r="E16" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9.999999999999998E-4</v>
       </c>
       <c r="F16" s="8">
@@ -2177,11 +2341,15 @@
         <v>0.99999999999999978</v>
       </c>
       <c r="G16" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.0000000000000233E-2</v>
       </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H16" s="11">
+        <f t="shared" si="2"/>
+        <v>5.0500000000000003E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B17" s="4">
         <v>25</v>
       </c>
@@ -2193,7 +2361,7 @@
         <v>1.28</v>
       </c>
       <c r="E17" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.2499999999999998E-3</v>
       </c>
       <c r="F17" s="4">
@@ -2201,11 +2369,15 @@
         <v>1.2499999999999998</v>
       </c>
       <c r="G17" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.4000000000000202E-2</v>
       </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H17" s="11">
+        <f t="shared" si="2"/>
+        <v>5.1200000000000002E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B18" s="4">
         <v>30</v>
       </c>
@@ -2217,7 +2389,7 @@
         <v>1.54</v>
       </c>
       <c r="E18" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.4999999999999998E-3</v>
       </c>
       <c r="F18" s="8">
@@ -2225,11 +2397,15 @@
         <v>1.4999999999999998</v>
       </c>
       <c r="G18" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.6666666666666842E-2</v>
       </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H18" s="11">
+        <f t="shared" si="2"/>
+        <v>5.1333333333333335E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B19" s="4">
         <v>35</v>
       </c>
@@ -2241,7 +2417,7 @@
         <v>1.77</v>
       </c>
       <c r="E19" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.7499999999999996E-3</v>
       </c>
       <c r="F19" s="4">
@@ -2249,11 +2425,15 @@
         <v>1.7499999999999996</v>
       </c>
       <c r="G19" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.1428571428571696E-2</v>
       </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H19" s="11">
+        <f t="shared" si="2"/>
+        <v>5.0571428571428573E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B20" s="4">
         <v>40</v>
       </c>
@@ -2265,7 +2445,7 @@
         <v>2.0499999999999998</v>
       </c>
       <c r="E20" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.9999999999999996E-3</v>
       </c>
       <c r="F20" s="8">
@@ -2273,11 +2453,15 @@
         <v>1.9999999999999996</v>
       </c>
       <c r="G20" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.500000000000014E-2</v>
       </c>
-    </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="H20" s="11">
+        <f t="shared" si="2"/>
+        <v>5.1249999999999997E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
         <v>23</v>
       </c>
@@ -2285,7 +2469,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" ht="16.2" x14ac:dyDescent="0.3">
       <c r="B24" s="5" t="s">
         <v>17</v>
       </c>
@@ -2293,7 +2477,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="16.8" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:8" ht="16.8" x14ac:dyDescent="0.35">
       <c r="B25" s="5" t="s">
         <v>24</v>
       </c>
@@ -2301,13 +2485,89 @@
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:8" ht="15.6" x14ac:dyDescent="0.35">
       <c r="B26" s="5" t="s">
         <v>25</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>20</v>
       </c>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B30" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" s="5"/>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B31" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C31" s="11">
+        <f>+AVERAGE(H13:H20)</f>
+        <v>5.0940178571428574E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B32" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C32" s="11">
+        <f>+F13/B13</f>
+        <v>4.9999999999999989E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B33" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C33" s="12">
+        <f>+(C31-C32)/C32</f>
+        <v>1.8803571428571701E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B34" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C34" s="5"/>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B37" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C37" s="5"/>
+    </row>
+    <row r="38" spans="2:3" ht="16.2" x14ac:dyDescent="0.3">
+      <c r="B38" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C38" s="5"/>
+    </row>
+    <row r="39" spans="2:3" ht="16.2" x14ac:dyDescent="0.3">
+      <c r="B39" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C39" s="5"/>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B40" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C40" s="8">
+        <f>+F16</f>
+        <v>0.99999999999999978</v>
+      </c>
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B41" s="8"/>
+      <c r="C41" s="5"/>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B42" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C42" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>